<commit_message>
feat(template): Supplier data-validation dropdown + remove dead FY_monthly_data.csv
Phase 4 of the data-migration review:
- build_template.py: add Supplier dropdown (13 canonical names, including
  long-form NISSEN CHEMITEC and APT (Thailand) so join keys match utils/
  supplier_aliases without normalization needed). Instructions sheet
  updated to mention the new dropdown.
- QA_Defects_Template.xlsx: regenerated with new Supplier DV attached to
  B5:B10000. Users now get an inline error when they type a typo instead
  of a silent broken join in the dashboard.
- tests/test_validation.py: 4 new regression tests asserting the Supplier
  DV is present and includes KSV + NISSEN CHEMITEC + APT (Thailand).
- Remove FY_monthly_data.csv (no code references; pre-dashboard FY data).
- Remove empty data/ directory (unused).

Test result: 40/40 pass (was 36/36 before this commit).
</commit_message>
<xml_diff>
--- a/QA_Defects_Template.xlsx
+++ b/QA_Defects_Template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📖 Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📚 Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="📖 Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Defects Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="📚 Reference" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -586,7 +586,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Use dropdowns for Group Part and Problem Mode</t>
+          <t>4. Use dropdowns for Group Part, Problem Mode, and Supplier</t>
         </is>
       </c>
     </row>
@@ -1031,12 +1031,15 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="C5:C10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Group Part" error="Please select a valid Group Part" promptTitle="Group Part" prompt="Select Group Part from dropdown" type="list">
       <formula1>"ELECTRIC &amp; ELEC.,PACKING,PIPING,PLASTIC,PRINTING,RAW MATERIAL,RUBBER,SHEET METAL,FOAM,SEALING,OTHERS"</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Problem Mode" error="Please select a valid Problem Mode" promptTitle="Problem Mode" prompt="Select Problem Mode from dropdown" type="list">
       <formula1>"APPEARANCE NG,PART MISTAKE,DIMENSION NG,FUNCTION NG,LEAK"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Supplier" error="Please select a valid Supplier from the dropdown" promptTitle="Supplier" prompt="Select Supplier from dropdown (typing a value not in list will fail validation)" type="list">
+      <formula1>"KSV,AKUSAN,NISSEN CHEMITEC,PARADISE,BTD,C.G.,TTS PLASTIC,SAMBO,DEM,APT (Thailand),SUPERFAST,SAM NEO,TECHNO ASSOCIATE"</formula1>
     </dataValidation>
     <dataValidation sqref="A5:A10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Date" error="Please enter a valid date (YYYY-MM-DD)" promptTitle="Date" prompt="Enter date as YYYY-MM-DD (e.g., 2026-08-31)" type="date" operator="between">
       <formula1>2020-01-01</formula1>

</xml_diff>